<commit_message>
fix: preserve hsr team observations
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbook_contract/hsr/hsr_endgame_dataset.xlsx
+++ b/tests/fixtures/workbook_contract/hsr/hsr_endgame_dataset.xlsx
@@ -1124,7 +1124,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>moc|all|1.0|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
+          <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
         </is>
       </c>
       <c r="AE2" t="n">
@@ -1137,12 +1137,12 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>moc|all|1.0|agent-alpha&gt;agent-beta&gt;agent-delta&gt;agent-gamma</t>
+          <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-delta&gt;agent-gamma</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>moc|all|1.0|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
+          <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>moc|all|1.0|agent-alpha&gt;agent-beta&gt;agent-delta&gt;agent-gamma</t>
+          <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-delta&gt;agent-gamma</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>moc|all|1.0|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
+          <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
         </is>
       </c>
       <c r="AE2" t="n">

</xml_diff>

<commit_message>
fix: distinguish hsr sample age and mirror evidence
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbook_contract/hsr/hsr_endgame_dataset.xlsx
+++ b/tests/fixtures/workbook_contract/hsr/hsr_endgame_dataset.xlsx
@@ -35,8 +35,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'character_usage_phase_latest'!$A$1:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'histograph_usage_long'!$A$1:$J$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'team_rank_raw'!$A$1:$AC$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'team_rank_dedup_ordered'!$A$1:$AF$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'team_rank_dedup_unordered'!$A$1:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'team_rank_dedup_ordered'!$A$1:$AG$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'team_rank_dedup_unordered'!$A$1:$AI$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'name_map'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'name_map_unresolved'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'prydwen_tier_current'!$A$1:$Y$2</definedName>
@@ -779,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -814,8 +814,9 @@
     <col width="36" customWidth="1" min="30" max="30"/>
     <col width="17" customWidth="1" min="31" max="31"/>
     <col width="28" customWidth="1" min="32" max="32"/>
-    <col width="36" customWidth="1" min="33" max="33"/>
-    <col width="28" customWidth="1" min="34" max="34"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
+    <col width="36" customWidth="1" min="34" max="34"/>
+    <col width="28" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -981,10 +982,15 @@
       </c>
       <c r="AG1" s="4" t="inlineStr">
         <is>
+          <t>merged_source_kinds</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
           <t>unordered_signature</t>
         </is>
       </c>
-      <c r="AH1" s="4" t="inlineStr">
+      <c r="AI1" s="4" t="inlineStr">
         <is>
           <t>ordered_signature_examples</t>
         </is>
@@ -1137,17 +1143,22 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
+          <t>hf_comps</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
           <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-delta&gt;agent-gamma</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>fixture-1|2026-07-12|moc|all|all|1.0|脱敏阶段|agent-alpha&gt;agent-beta&gt;agent-gamma&gt;agent-delta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AH2"/>
+  <autoFilter ref="A1:AI2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3838,7 +3849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3873,6 +3884,7 @@
     <col width="36" customWidth="1" min="30" max="30"/>
     <col width="17" customWidth="1" min="31" max="31"/>
     <col width="28" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4036,6 +4048,11 @@
           <t>merged_source_files</t>
         </is>
       </c>
+      <c r="AG1" s="4" t="inlineStr">
+        <is>
+          <t>merged_source_kinds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4182,9 +4199,14 @@
           <t>fixture/teams.json</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>hf_comps</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF2"/>
+  <autoFilter ref="A1:AG2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>